<commit_message>
Revert "Merge branch 'Principal' of https://github.com/Shizars/Proyecto-ing-soft-1-y-2 into Principal"
This reverts commit fb1c45edebbab94b756670a67698e29012b1fa4e, reversing
changes made to 267c8d87b8635a257d8f101f92421717e05d5911.
</commit_message>
<xml_diff>
--- a/INCREMENTO 2/Burn-down.xlsx
+++ b/INCREMENTO 2/Burn-down.xlsx
@@ -9,7 +9,7 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="LFzCVT5HlJTl1MBarwUB7tFN2WUuqGyTK9pZGwQUCfY="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId5" roundtripDataChecksum="3G+M+f8GiXOUhMUf438CylTAQPK0nlxAIox20duR4hE="/>
     </ext>
   </extLst>
 </workbook>
@@ -84,17 +84,18 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
     <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="4" fontId="1" numFmtId="164" xfId="0" applyFill="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="0" fillId="4" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFill="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="5" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="5" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -363,10 +364,10 @@
         <v>45901.0</v>
       </c>
       <c r="B3" s="4">
-        <v>698.0</v>
+        <v>690.0</v>
       </c>
       <c r="C3" s="4">
-        <v>852.0</v>
+        <v>890.0</v>
       </c>
     </row>
     <row r="4">
@@ -374,10 +375,10 @@
         <v>45902.0</v>
       </c>
       <c r="B4" s="4">
-        <v>698.0</v>
+        <v>690.0</v>
       </c>
       <c r="C4" s="4">
-        <v>825.0</v>
+        <v>835.0</v>
       </c>
     </row>
     <row r="5">
@@ -385,9 +386,9 @@
         <v>45903.0</v>
       </c>
       <c r="B5" s="4">
-        <v>698.0</v>
-      </c>
-      <c r="C5" s="5">
+        <v>690.0</v>
+      </c>
+      <c r="C5" s="4">
         <v>793.0</v>
       </c>
     </row>
@@ -396,9 +397,9 @@
         <v>45904.0</v>
       </c>
       <c r="B6" s="4">
-        <v>698.0</v>
-      </c>
-      <c r="C6" s="5">
+        <v>690.0</v>
+      </c>
+      <c r="C6" s="4">
         <v>771.0</v>
       </c>
     </row>
@@ -406,10 +407,10 @@
       <c r="A7" s="3">
         <v>45905.0</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="4">
         <v>690.0</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="4">
         <v>715.0</v>
       </c>
     </row>
@@ -417,10 +418,10 @@
       <c r="A8" s="3">
         <v>45906.0</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="4">
         <v>690.0</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="4">
         <v>625.0</v>
       </c>
     </row>
@@ -429,9 +430,9 @@
         <v>45907.0</v>
       </c>
       <c r="B9" s="4">
-        <v>658.0</v>
-      </c>
-      <c r="C9" s="5">
+        <v>683.0</v>
+      </c>
+      <c r="C9" s="4">
         <v>596.0</v>
       </c>
     </row>
@@ -440,9 +441,9 @@
         <v>45908.0</v>
       </c>
       <c r="B10" s="4">
-        <v>631.0</v>
-      </c>
-      <c r="C10" s="5">
+        <v>578.0</v>
+      </c>
+      <c r="C10" s="4">
         <v>531.0</v>
       </c>
     </row>
@@ -451,9 +452,9 @@
         <v>45909.0</v>
       </c>
       <c r="B11" s="4">
-        <v>582.0</v>
-      </c>
-      <c r="C11" s="5">
+        <v>534.0</v>
+      </c>
+      <c r="C11" s="4">
         <v>492.0</v>
       </c>
     </row>
@@ -462,9 +463,9 @@
         <v>45910.0</v>
       </c>
       <c r="B12" s="4">
-        <v>512.0</v>
-      </c>
-      <c r="C12" s="5">
+        <v>501.0</v>
+      </c>
+      <c r="C12" s="4">
         <v>473.0</v>
       </c>
     </row>
@@ -472,10 +473,10 @@
       <c r="A13" s="3">
         <v>45911.0</v>
       </c>
-      <c r="B13" s="5">
+      <c r="B13" s="4">
         <v>486.0</v>
       </c>
-      <c r="C13" s="5">
+      <c r="C13" s="4">
         <v>458.0</v>
       </c>
     </row>
@@ -483,10 +484,10 @@
       <c r="A14" s="3">
         <v>45912.0</v>
       </c>
-      <c r="B14" s="5">
+      <c r="B14" s="4">
         <v>453.0</v>
       </c>
-      <c r="C14" s="5">
+      <c r="C14" s="4">
         <v>412.0</v>
       </c>
     </row>
@@ -494,10 +495,10 @@
       <c r="A15" s="3">
         <v>45913.0</v>
       </c>
-      <c r="B15" s="5">
+      <c r="B15" s="4">
         <v>421.0</v>
       </c>
-      <c r="C15" s="5">
+      <c r="C15" s="4">
         <v>388.0</v>
       </c>
     </row>
@@ -505,10 +506,10 @@
       <c r="A16" s="3">
         <v>45914.0</v>
       </c>
-      <c r="B16" s="5">
+      <c r="B16" s="4">
         <v>394.0</v>
       </c>
-      <c r="C16" s="5">
+      <c r="C16" s="4">
         <v>356.0</v>
       </c>
     </row>
@@ -516,10 +517,10 @@
       <c r="A17" s="3">
         <v>45915.0</v>
       </c>
-      <c r="B17" s="5">
+      <c r="B17" s="4">
         <v>375.0</v>
       </c>
-      <c r="C17" s="5">
+      <c r="C17" s="4">
         <v>328.0</v>
       </c>
     </row>
@@ -527,10 +528,10 @@
       <c r="A18" s="3">
         <v>45916.0</v>
       </c>
-      <c r="B18" s="5">
+      <c r="B18" s="4">
         <v>349.0</v>
       </c>
-      <c r="C18" s="5">
+      <c r="C18" s="4">
         <v>298.0</v>
       </c>
     </row>
@@ -538,10 +539,10 @@
       <c r="A19" s="3">
         <v>45917.0</v>
       </c>
-      <c r="B19" s="5">
+      <c r="B19" s="4">
         <v>328.0</v>
       </c>
-      <c r="C19" s="5">
+      <c r="C19" s="4">
         <v>278.0</v>
       </c>
     </row>
@@ -549,10 +550,10 @@
       <c r="A20" s="3">
         <v>45918.0</v>
       </c>
-      <c r="B20" s="5">
+      <c r="B20" s="4">
         <v>290.0</v>
       </c>
-      <c r="C20" s="5">
+      <c r="C20" s="4">
         <v>254.0</v>
       </c>
     </row>
@@ -560,10 +561,10 @@
       <c r="A21" s="3">
         <v>45919.0</v>
       </c>
-      <c r="B21" s="5">
+      <c r="B21" s="4">
         <v>290.0</v>
       </c>
-      <c r="C21" s="5">
+      <c r="C21" s="4">
         <v>221.0</v>
       </c>
     </row>
@@ -571,10 +572,10 @@
       <c r="A22" s="3">
         <v>45920.0</v>
       </c>
-      <c r="B22" s="5">
+      <c r="B22" s="4">
         <v>267.0</v>
       </c>
-      <c r="C22" s="5">
+      <c r="C22" s="4">
         <v>198.0</v>
       </c>
     </row>
@@ -582,10 +583,10 @@
       <c r="A23" s="3">
         <v>45921.0</v>
       </c>
-      <c r="B23" s="5">
+      <c r="B23" s="4">
         <v>238.0</v>
       </c>
-      <c r="C23" s="5">
+      <c r="C23" s="4">
         <v>180.0</v>
       </c>
     </row>
@@ -593,10 +594,10 @@
       <c r="A24" s="3">
         <v>45922.0</v>
       </c>
-      <c r="B24" s="5">
+      <c r="B24" s="4">
         <v>204.0</v>
       </c>
-      <c r="C24" s="5">
+      <c r="C24" s="4">
         <v>167.0</v>
       </c>
     </row>
@@ -604,10 +605,10 @@
       <c r="A25" s="3">
         <v>45923.0</v>
       </c>
-      <c r="B25" s="5">
+      <c r="B25" s="4">
         <v>181.0</v>
       </c>
-      <c r="C25" s="5">
+      <c r="C25" s="4">
         <v>151.0</v>
       </c>
     </row>
@@ -615,10 +616,10 @@
       <c r="A26" s="3">
         <v>45924.0</v>
       </c>
-      <c r="B26" s="5">
+      <c r="B26" s="4">
         <v>164.0</v>
       </c>
-      <c r="C26" s="5">
+      <c r="C26" s="4">
         <v>135.0</v>
       </c>
     </row>
@@ -626,10 +627,10 @@
       <c r="A27" s="3">
         <v>45925.0</v>
       </c>
-      <c r="B27" s="5">
+      <c r="B27" s="4">
         <v>142.0</v>
       </c>
-      <c r="C27" s="5">
+      <c r="C27" s="4">
         <v>121.0</v>
       </c>
     </row>
@@ -637,10 +638,10 @@
       <c r="A28" s="3">
         <v>45926.0</v>
       </c>
-      <c r="B28" s="5">
+      <c r="B28" s="4">
         <v>107.0</v>
       </c>
-      <c r="C28" s="5">
+      <c r="C28" s="4">
         <v>105.0</v>
       </c>
     </row>
@@ -648,10 +649,10 @@
       <c r="A29" s="3">
         <v>45927.0</v>
       </c>
-      <c r="B29" s="5">
+      <c r="B29" s="4">
         <v>82.0</v>
       </c>
-      <c r="C29" s="5">
+      <c r="C29" s="4">
         <v>87.0</v>
       </c>
     </row>
@@ -659,10 +660,10 @@
       <c r="A30" s="3">
         <v>45928.0</v>
       </c>
-      <c r="B30" s="5">
+      <c r="B30" s="4">
         <v>60.0</v>
       </c>
-      <c r="C30" s="5">
+      <c r="C30" s="4">
         <v>64.0</v>
       </c>
     </row>
@@ -670,10 +671,10 @@
       <c r="A31" s="3">
         <v>45929.0</v>
       </c>
-      <c r="B31" s="5">
+      <c r="B31" s="4">
         <v>41.0</v>
       </c>
-      <c r="C31" s="5">
+      <c r="C31" s="4">
         <v>43.0</v>
       </c>
     </row>
@@ -681,10 +682,10 @@
       <c r="A32" s="3">
         <v>45930.0</v>
       </c>
-      <c r="B32" s="5">
+      <c r="B32" s="4">
         <v>12.0</v>
       </c>
-      <c r="C32" s="5">
+      <c r="C32" s="4">
         <v>29.0</v>
       </c>
     </row>
@@ -692,11 +693,33 @@
       <c r="A33" s="3">
         <v>45931.0</v>
       </c>
-      <c r="B33" s="5">
+      <c r="B33" s="4">
         <v>6.0</v>
       </c>
-      <c r="C33" s="5">
+      <c r="C33" s="4">
         <v>16.0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3">
+        <v>45932.0</v>
+      </c>
+      <c r="B34" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="C34" s="4">
+        <v>9.0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3">
+        <v>45933.0</v>
+      </c>
+      <c r="B35" s="4">
+        <v>0.0</v>
+      </c>
+      <c r="C35" s="4">
+        <v>0.0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>